<commit_message>
Ajusta eliminacoes nas ligas eliminacao
</commit_message>
<xml_diff>
--- a/liga_eliminacao/datasets_liga_eliminacao/Pontuacoes_Por_Rodada_Liga_Eliminacao.xlsx
+++ b/liga_eliminacao/datasets_liga_eliminacao/Pontuacoes_Por_Rodada_Liga_Eliminacao.xlsx
@@ -76,7 +76,7 @@
     <t>Rodada 19</t>
   </si>
   <si>
-    <t>Parcial Rodada 1</t>
+    <t>Parcial Rodada 2</t>
   </si>
   <si>
     <t>time_id</t>
@@ -612,10 +612,10 @@
         <v>22</v>
       </c>
       <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="V2">
-        <v>68.06</v>
+        <v>68.06005859375</v>
+      </c>
+      <c r="D2">
+        <v>68.06005859375</v>
       </c>
     </row>
     <row r="3" spans="1:22">
@@ -626,10 +626,10 @@
         <v>23</v>
       </c>
       <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="V3">
-        <v>53.66</v>
+        <v>53.659912109375</v>
+      </c>
+      <c r="D3">
+        <v>53.659912109375</v>
       </c>
     </row>
     <row r="4" spans="1:22">
@@ -640,10 +640,10 @@
         <v>24</v>
       </c>
       <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="V4">
-        <v>66.86</v>
+        <v>66.85986328125</v>
+      </c>
+      <c r="D4">
+        <v>66.85986328125</v>
       </c>
     </row>
     <row r="5" spans="1:22">
@@ -654,9 +654,9 @@
         <v>25</v>
       </c>
       <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="V5">
+        <v>70</v>
+      </c>
+      <c r="D5">
         <v>70</v>
       </c>
     </row>
@@ -668,10 +668,10 @@
         <v>26</v>
       </c>
       <c r="C6">
-        <v>0</v>
-      </c>
-      <c r="V6">
-        <v>58.96</v>
+        <v>58.9599609375</v>
+      </c>
+      <c r="D6">
+        <v>58.9599609375</v>
       </c>
     </row>
     <row r="7" spans="1:22">
@@ -682,10 +682,10 @@
         <v>27</v>
       </c>
       <c r="C7">
-        <v>0</v>
-      </c>
-      <c r="V7">
-        <v>57.45</v>
+        <v>57.449951171875</v>
+      </c>
+      <c r="D7">
+        <v>57.449951171875</v>
       </c>
     </row>
     <row r="8" spans="1:22">
@@ -696,10 +696,10 @@
         <v>28</v>
       </c>
       <c r="C8">
-        <v>0</v>
-      </c>
-      <c r="V8">
-        <v>68.06</v>
+        <v>68.06005859375</v>
+      </c>
+      <c r="D8">
+        <v>68.06005859375</v>
       </c>
     </row>
     <row r="9" spans="1:22">
@@ -710,10 +710,10 @@
         <v>29</v>
       </c>
       <c r="C9">
-        <v>0</v>
-      </c>
-      <c r="V9">
-        <v>47.86</v>
+        <v>47.860107421875</v>
+      </c>
+      <c r="D9">
+        <v>47.860107421875</v>
       </c>
     </row>
     <row r="10" spans="1:22">
@@ -724,10 +724,10 @@
         <v>30</v>
       </c>
       <c r="C10">
-        <v>0</v>
-      </c>
-      <c r="V10">
-        <v>64.56</v>
+        <v>64.56005859375</v>
+      </c>
+      <c r="D10">
+        <v>64.56005859375</v>
       </c>
     </row>
     <row r="11" spans="1:22">
@@ -738,10 +738,10 @@
         <v>31</v>
       </c>
       <c r="C11">
-        <v>0</v>
-      </c>
-      <c r="V11">
-        <v>44.26</v>
+        <v>44.260009765625</v>
+      </c>
+      <c r="D11">
+        <v>44.260009765625</v>
       </c>
     </row>
     <row r="12" spans="1:22">
@@ -752,10 +752,10 @@
         <v>32</v>
       </c>
       <c r="C12">
-        <v>0</v>
-      </c>
-      <c r="V12">
-        <v>61.56</v>
+        <v>61.56005859375</v>
+      </c>
+      <c r="D12">
+        <v>61.56005859375</v>
       </c>
     </row>
     <row r="13" spans="1:22">
@@ -766,10 +766,10 @@
         <v>33</v>
       </c>
       <c r="C13">
-        <v>0</v>
-      </c>
-      <c r="V13">
-        <v>84.86</v>
+        <v>84.85986328125</v>
+      </c>
+      <c r="D13">
+        <v>84.85986328125</v>
       </c>
     </row>
     <row r="14" spans="1:22">
@@ -780,10 +780,7 @@
         <v>34</v>
       </c>
       <c r="C14">
-        <v>0</v>
-      </c>
-      <c r="V14">
-        <v>42.96</v>
+        <v>42.9599609375</v>
       </c>
     </row>
     <row r="15" spans="1:22">
@@ -794,10 +791,10 @@
         <v>35</v>
       </c>
       <c r="C15">
-        <v>0</v>
-      </c>
-      <c r="V15">
-        <v>74.06</v>
+        <v>74.06005859375</v>
+      </c>
+      <c r="D15">
+        <v>74.06005859375</v>
       </c>
     </row>
     <row r="16" spans="1:22">
@@ -808,13 +805,13 @@
         <v>36</v>
       </c>
       <c r="C16">
-        <v>0</v>
-      </c>
-      <c r="V16">
-        <v>54.6</v>
-      </c>
-    </row>
-    <row r="17" spans="1:22">
+        <v>54.60009765625</v>
+      </c>
+      <c r="D16">
+        <v>54.60009765625</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
       <c r="A17" s="1">
         <v>14124559</v>
       </c>
@@ -822,13 +819,13 @@
         <v>37</v>
       </c>
       <c r="C17">
-        <v>0</v>
-      </c>
-      <c r="V17">
-        <v>84.26000000000001</v>
-      </c>
-    </row>
-    <row r="18" spans="1:22">
+        <v>84.259765625</v>
+      </c>
+      <c r="D17">
+        <v>84.259765625</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
       <c r="A18" s="1">
         <v>18223508</v>
       </c>
@@ -836,13 +833,13 @@
         <v>38</v>
       </c>
       <c r="C18">
-        <v>0</v>
-      </c>
-      <c r="V18">
         <v>59.25</v>
       </c>
-    </row>
-    <row r="19" spans="1:22">
+      <c r="D18">
+        <v>59.25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
       <c r="A19" s="1">
         <v>18344271</v>
       </c>
@@ -850,13 +847,13 @@
         <v>39</v>
       </c>
       <c r="C19">
-        <v>0</v>
-      </c>
-      <c r="V19">
-        <v>54.16</v>
-      </c>
-    </row>
-    <row r="20" spans="1:22">
+        <v>54.159912109375</v>
+      </c>
+      <c r="D19">
+        <v>54.159912109375</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
       <c r="A20" s="1">
         <v>18642587</v>
       </c>
@@ -864,13 +861,13 @@
         <v>40</v>
       </c>
       <c r="C20">
-        <v>0</v>
-      </c>
-      <c r="V20">
-        <v>63.9</v>
-      </c>
-    </row>
-    <row r="21" spans="1:22">
+        <v>63.89990234375</v>
+      </c>
+      <c r="D20">
+        <v>63.89990234375</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
       <c r="A21" s="1">
         <v>18661583</v>
       </c>
@@ -878,13 +875,13 @@
         <v>41</v>
       </c>
       <c r="C21">
-        <v>0</v>
-      </c>
-      <c r="V21">
-        <v>50.26</v>
-      </c>
-    </row>
-    <row r="22" spans="1:22">
+        <v>50.260009765625</v>
+      </c>
+      <c r="D21">
+        <v>50.260009765625</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
       <c r="A22" s="1">
         <v>19033717</v>
       </c>
@@ -892,13 +889,13 @@
         <v>42</v>
       </c>
       <c r="C22">
-        <v>0</v>
-      </c>
-      <c r="V22">
-        <v>73.95999999999999</v>
-      </c>
-    </row>
-    <row r="23" spans="1:22">
+        <v>73.9599609375</v>
+      </c>
+      <c r="D22">
+        <v>73.9599609375</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
       <c r="A23" s="1">
         <v>20696550</v>
       </c>
@@ -906,13 +903,13 @@
         <v>43</v>
       </c>
       <c r="C23">
-        <v>0</v>
-      </c>
-      <c r="V23">
-        <v>72.7</v>
-      </c>
-    </row>
-    <row r="24" spans="1:22">
+        <v>72.7001953125</v>
+      </c>
+      <c r="D23">
+        <v>72.7001953125</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
       <c r="A24" s="1">
         <v>24468241</v>
       </c>
@@ -920,13 +917,13 @@
         <v>44</v>
       </c>
       <c r="C24">
-        <v>0</v>
-      </c>
-      <c r="V24">
-        <v>57.6</v>
-      </c>
-    </row>
-    <row r="25" spans="1:22">
+        <v>57.60009765625</v>
+      </c>
+      <c r="D24">
+        <v>57.60009765625</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
       <c r="A25" s="1">
         <v>24856400</v>
       </c>
@@ -934,13 +931,13 @@
         <v>45</v>
       </c>
       <c r="C25">
-        <v>0</v>
-      </c>
-      <c r="V25">
-        <v>64.7</v>
-      </c>
-    </row>
-    <row r="26" spans="1:22">
+        <v>64.7001953125</v>
+      </c>
+      <c r="D25">
+        <v>64.7001953125</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
       <c r="A26" s="1">
         <v>25565675</v>
       </c>
@@ -948,13 +945,13 @@
         <v>46</v>
       </c>
       <c r="C26">
-        <v>0</v>
-      </c>
-      <c r="V26">
-        <v>44.06</v>
-      </c>
-    </row>
-    <row r="27" spans="1:22">
+        <v>44.06005859375</v>
+      </c>
+      <c r="D26">
+        <v>44.06005859375</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
       <c r="A27" s="1">
         <v>25811332</v>
       </c>
@@ -962,13 +959,13 @@
         <v>47</v>
       </c>
       <c r="C27">
-        <v>0</v>
-      </c>
-      <c r="V27">
         <v>49</v>
       </c>
-    </row>
-    <row r="28" spans="1:22">
+      <c r="D27">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
       <c r="A28" s="1">
         <v>28741323</v>
       </c>
@@ -976,13 +973,13 @@
         <v>48</v>
       </c>
       <c r="C28">
-        <v>0</v>
-      </c>
-      <c r="V28">
-        <v>61.96</v>
-      </c>
-    </row>
-    <row r="29" spans="1:22">
+        <v>61.9599609375</v>
+      </c>
+      <c r="D28">
+        <v>61.9599609375</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
       <c r="A29" s="1">
         <v>29228373</v>
       </c>
@@ -990,13 +987,13 @@
         <v>49</v>
       </c>
       <c r="C29">
-        <v>0</v>
-      </c>
-      <c r="V29">
-        <v>60.16</v>
-      </c>
-    </row>
-    <row r="30" spans="1:22">
+        <v>60.159912109375</v>
+      </c>
+      <c r="D29">
+        <v>60.159912109375</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
       <c r="A30" s="1">
         <v>44810918</v>
       </c>
@@ -1004,13 +1001,13 @@
         <v>50</v>
       </c>
       <c r="C30">
-        <v>0</v>
-      </c>
-      <c r="V30">
-        <v>62.56</v>
-      </c>
-    </row>
-    <row r="31" spans="1:22">
+        <v>62.56005859375</v>
+      </c>
+      <c r="D30">
+        <v>62.56005859375</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
       <c r="A31" s="1">
         <v>47544767</v>
       </c>
@@ -1018,13 +1015,13 @@
         <v>51</v>
       </c>
       <c r="C31">
-        <v>0</v>
-      </c>
-      <c r="V31">
-        <v>73.76000000000001</v>
-      </c>
-    </row>
-    <row r="32" spans="1:22">
+        <v>73.759765625</v>
+      </c>
+      <c r="D31">
+        <v>73.759765625</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
       <c r="A32" s="1">
         <v>48498051</v>
       </c>
@@ -1032,13 +1029,13 @@
         <v>52</v>
       </c>
       <c r="C32">
-        <v>0</v>
-      </c>
-      <c r="V32">
-        <v>64.56</v>
-      </c>
-    </row>
-    <row r="33" spans="1:22">
+        <v>64.56005859375</v>
+      </c>
+      <c r="D32">
+        <v>64.56005859375</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
       <c r="A33" s="1">
         <v>51010813</v>
       </c>
@@ -1046,10 +1043,10 @@
         <v>53</v>
       </c>
       <c r="C33">
-        <v>0</v>
-      </c>
-      <c r="V33">
-        <v>47.86</v>
+        <v>47.860107421875</v>
+      </c>
+      <c r="D33">
+        <v>47.860107421875</v>
       </c>
     </row>
   </sheetData>

</xml_diff>